<commit_message>
Elevate Bookend doctrine to foundational across canon
Add the three foundational principles, Bookend Rule (PJ owns the Entry
Surface and the Repository), Agnostic Middle Rule (content-agnostic but
governance-aware), and the Runtime Contract to all three artifacts:
- PUBLICLOGIC_CANON.md -> V1.1; new §1 principles + Bookend/Agnostic
  Middle/Runtime Contract; §16 category sharpened to "governed
  transitions between two immutable guarantees".
- PublicLogic-Canon.xlsx -> cover gains the three principles; Runtime
  Line tab gains a Bookend note.
- PublicLogic_Series1_Final_Workbook.xlsx -> 01_Core_Doctrine gains
  Bookend Rule and Agnostic Middle Rule rows (lossless edit).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VAv7tVCy2hbSMpZ9X88jpW
</commit_message>
<xml_diff>
--- a/publiclogic/docs/canon/PublicLogic-Canon.xlsx
+++ b/publiclogic/docs/canon/PublicLogic-Canon.xlsx
@@ -76,15 +76,15 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="0040554D"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="20"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="0040554D"/>
-      <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
@@ -116,12 +116,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3A2E"/>
+        <fgColor rgb="00EAF1ED"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EAF1ED"/>
+        <fgColor rgb="001F3A2E"/>
       </patternFill>
     </fill>
     <fill>
@@ -181,7 +181,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -207,37 +207,40 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -612,7 +615,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B34"/>
+  <dimension ref="A1:B41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -671,266 +674,330 @@
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Tabs in this workbook</t>
+          <t>The three foundational principles</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Tab</t>
+          <t>#</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Principle</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>00 Index</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Cover, final doctrine, distilled rulings, tab index, legend.</t>
+          <t>CaseSpace is the only primitive.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>01 Position</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>What we are, what we are not, relationship to larger governance systems, taglines.</t>
+          <t>PuddleJumper owns the two guarantees: Entry and Repository.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>02 Runtime Line</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>The canonical FORM→ARCHIEVE sequence, one row per stage.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>03 Primitives</t>
-        </is>
-      </c>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>Core runtime primitives and the OPS preset modules.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="7" t="inlineStr">
-        <is>
-          <t>04 Rulings</t>
-        </is>
-      </c>
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>The four LOCKED rulings. 🔒</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>05 CaseSpace Model</t>
-        </is>
-      </c>
-      <c r="B19" s="8" t="inlineStr">
-        <is>
-          <t>Type field, standing vs closing, object model, lifecycles, nesting.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>06 Conflict Types</t>
-        </is>
-      </c>
-      <c r="B20" s="8" t="inlineStr">
-        <is>
-          <t>The five conflicts, their source, detection, and routing.</t>
+          <t>The middle is content-agnostic but governance-aware.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="120" customHeight="1">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>Bookend Rule: PJ owns the Entry Surface (received → logged) and the Repository (closed → sealed → rolled up). Everything between belongs to the operator — content-agnostic, not unconstrained. Category: governed transitions between two immutable guarantees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Tabs in this workbook</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Tab</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Description</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>07 Type Catalogue</t>
+          <t>00 Index</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>Leaf types and container types.</t>
+          <t>Cover, final doctrine, distilled rulings, tab index, legend.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>08 Type=Skin</t>
+          <t>01 Position</t>
         </is>
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>Type-as-skin binding and the authoring rule.</t>
+          <t>What we are, what we are not, relationship to larger governance systems, taglines.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>09 Canon Laws</t>
+          <t>02 Runtime Line</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>The seven canon laws.</t>
+          <t>The canonical FORM→ARCHIEVE sequence, one row per stage.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>10 Templates</t>
+          <t>03 Primitives</t>
         </is>
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>Module Maker template set (STAY MUNI BIZ GRANT LIVE HOME).</t>
+          <t>Core runtime primitives and the OPS preset modules.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>11 Vocabulary</t>
+          <t>04 Rulings</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>Canon terms, user-facing labels, retired terms.</t>
+          <t>The four LOCKED rulings. 🔒</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>12 VAULT</t>
+          <t>05 CaseSpace Model</t>
         </is>
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>VAULT doctrine — five principles and their enforcing mechanism.</t>
+          <t>Type field, standing vs closing, object model, lifecycles, nesting.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>13 Proven vs Open</t>
+          <t>06 Conflict Types</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>What is proven at 54cdaa5 and what remains open. ◻</t>
+          <t>The five conflicts, their source, detection, and routing.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>14 GTM</t>
+          <t>07 Type Catalogue</t>
         </is>
       </c>
       <c r="B28" s="8" t="inlineStr">
         <is>
-          <t>Commercial packaging — NON-DOCTRINE, fenced. ⚠</t>
+          <t>Leaf types and container types.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>15 Build Order</t>
+          <t>08 Type=Skin</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>Sequence of embodiment: STAY → MUNI → LIVE support → BIZ/GRANT/HOME.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>Legend</t>
+          <t>Type-as-skin binding and the authoring rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>09 Canon Laws</t>
+        </is>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>The seven canon laws.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>10 Templates</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>Module Maker template set (STAY MUNI BIZ GRANT LIVE HOME).</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>🔒 Locked</t>
+          <t>11 Vocabulary</t>
         </is>
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>Settled doctrine — not an open question.</t>
+          <t>Canon terms, user-facing labels, retired terms.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>◻ Open call</t>
+          <t>12 VAULT</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>Unresolved decision, tracked as open.</t>
+          <t>VAULT doctrine — five principles and their enforcing mechanism.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
+          <t>13 Proven vs Open</t>
+        </is>
+      </c>
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>What is proven at 54cdaa5 and what remains open. ◻</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>14 GTM</t>
+        </is>
+      </c>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>Commercial packaging — NON-DOCTRINE, fenced. ⚠</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>15 Build Order</t>
+        </is>
+      </c>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>Sequence of embodiment: STAY → MUNI → LIVE support → BIZ/GRANT/HOME.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="22" customHeight="1">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Legend</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>🔒 Locked</t>
+        </is>
+      </c>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>Settled doctrine — not an open question.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>◻ Open call</t>
+        </is>
+      </c>
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>Unresolved decision, tracked as open.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
           <t>⚠ Non-doctrine</t>
         </is>
       </c>
-      <c r="B34" s="8" t="inlineStr">
+      <c r="B41" s="8" t="inlineStr">
         <is>
           <t>Commercial packaging, subject to change.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="11">
     <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A38:B38"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A19:B19"/>
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A17:B17"/>
     <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A31:B31"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A12:B12"/>
   </mergeCells>
@@ -953,14 +1020,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>09 · Canon Laws</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>The abstraction is the law; the tools are swappable.</t>
         </is>
@@ -1089,21 +1156,21 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>10 · Templates (Module Maker set)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>Each template = one standing parent + child leaf cases. Maturity ∈ {proven · scaffolded · framed · deferred}.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>STAY is the first fully embodied proof lane; MUNI is scaffolded alongside it; the rest are template families at lower maturity. Maturity labels track embodiment, not value.</t>
         </is>
@@ -1669,14 +1736,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>11 · Vocabulary</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>Canon terms, the labels users see, and what is retired.</t>
         </is>
@@ -1804,48 +1871,48 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="16" t="inlineStr">
+      <c r="A19" s="17" t="inlineStr">
         <is>
           <t>Cockpit Module</t>
         </is>
       </c>
-      <c r="B19" s="17" t="inlineStr">
+      <c r="B19" s="18" t="inlineStr">
         <is>
           <t>retired — never use as a live term</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="16" t="inlineStr">
+      <c r="A20" s="17" t="inlineStr">
         <is>
           <t>Open Cockpit</t>
         </is>
       </c>
-      <c r="B20" s="17" t="inlineStr">
+      <c r="B20" s="18" t="inlineStr">
         <is>
           <t>retired — never use as a live term</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="16" t="inlineStr">
+      <c r="A21" s="17" t="inlineStr">
         <is>
           <t>Build My Cockpit</t>
         </is>
       </c>
-      <c r="B21" s="17" t="inlineStr">
+      <c r="B21" s="18" t="inlineStr">
         <is>
           <t>retired — never use as a live term</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="16" t="inlineStr">
+      <c r="A22" s="17" t="inlineStr">
         <is>
           <t>LogicOS</t>
         </is>
       </c>
-      <c r="B22" s="17" t="inlineStr">
+      <c r="B22" s="18" t="inlineStr">
         <is>
           <t>retired — never use as a live term</t>
         </is>
@@ -1880,21 +1947,21 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>12 · VAULT (doctrine)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>VAULT = Verification · Authority · Utility · Legitimacy · Transfer. Doctrine, not a stage.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="45" customHeight="1">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>Enforced by CAL gates and the append-only audit stream. VAULT is doctrine, not a pipeline stage. V/A/L/T are settled; the U (Utility) mechanism is a proposed, not-yet-ratified mapping (see note below).</t>
         </is>
@@ -1967,22 +2034,22 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="B9" s="16" t="inlineStr">
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t>Utility</t>
         </is>
       </c>
-      <c r="C9" s="18" t="inlineStr">
+      <c r="C9" s="19" t="inlineStr">
         <is>
           <t>The record is usable for the work it governs — proposed enforcement: skin-defined required fields and structured FORM intake make the record complete and retrievable, with the missing_evidence CAL conflict blocking close until the usable record is whole. [ILLUSTRATIVE — proposed, not yet ratified.]</t>
         </is>
       </c>
-      <c r="D9" s="18" t="inlineStr">
+      <c r="D9" s="19" t="inlineStr">
         <is>
           <t>◻ proposed</t>
         </is>
@@ -2033,7 +2100,7 @@
       </c>
     </row>
     <row r="13" ht="90" customHeight="1">
-      <c r="A13" s="15" t="inlineStr">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>Utility (U) mechanism is fenced exactly like the Type Catalogue: the PRINCIPLE is canon; the enforcing mechanism above is a proposed mapping derived from existing primitives (skin schema + FORM intake + missing_evidence CAL conflict), routed through propose-then-ratify before it becomes locked doctrine. Until ratified, treat the U mechanism as TBD, not settled.</t>
         </is>
@@ -2065,14 +2132,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>13 · Proven vs Open</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>Everything reconciles to runtime commit 54cdaa5 (origin/logic-commons-v1).</t>
         </is>
@@ -2335,21 +2402,21 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="19" t="inlineStr">
+      <c r="A1" s="20" t="inlineStr">
         <is>
           <t>14 · GTM  ⚠ NON-DOCTRINE</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>Commercial packaging. Read in light of the banner below.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="26" customHeight="1">
-      <c r="A4" s="20" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>NOT DOCTRINE — commercial packaging, subject to change.</t>
         </is>
@@ -2363,17 +2430,17 @@
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="21" t="inlineStr">
+      <c r="A7" s="22" t="inlineStr">
         <is>
           <t>Lane</t>
         </is>
       </c>
-      <c r="B7" s="21" t="inlineStr">
+      <c r="B7" s="22" t="inlineStr">
         <is>
           <t>From</t>
         </is>
       </c>
-      <c r="C7" s="21" t="inlineStr"/>
+      <c r="C7" s="22" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -2435,34 +2502,34 @@
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="21" t="inlineStr">
+      <c r="A14" s="22" t="inlineStr">
         <is>
           <t>Offer</t>
         </is>
       </c>
-      <c r="B14" s="21" t="inlineStr">
+      <c r="B14" s="22" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
-      <c r="C14" s="21" t="inlineStr">
+      <c r="C14" s="22" t="inlineStr">
         <is>
           <t>What</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="inlineStr">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>Self-Build Template</t>
         </is>
       </c>
-      <c r="B15" s="18" t="inlineStr">
+      <c r="B15" s="19" t="inlineStr">
         <is>
           <t>$29–$49/mo</t>
         </is>
       </c>
-      <c r="C15" s="18" t="inlineStr">
+      <c r="C15" s="19" t="inlineStr">
         <is>
           <t>User builds CaseSpace templates from a library. ⚠ FLAGGED: requires un-built self-serve software; conflicts with the proven path of productized service, not platform. Aspirational, not committed.</t>
         </is>
@@ -2537,7 +2604,7 @@
       </c>
     </row>
     <row r="21" ht="60" customHeight="1">
-      <c r="A21" s="15" t="inlineStr">
+      <c r="A21" s="16" t="inlineStr">
         <is>
           <t>The near-term motion is productized service proven on yourself first (Kendall Pond), sold to one customer, delivered and timed — not a self-serve platform launch.</t>
         </is>
@@ -2573,21 +2640,21 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>15 · Build Order</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>The sequence of embodiment. Build the primitives once; embody the lanes in order.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="45" customHeight="1">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>Order reflects proof maturity and the productized-service motion (prove on yourself first, then sell one). It is a build sequence, not a value ranking.</t>
         </is>
@@ -2704,7 +2771,7 @@
       </c>
     </row>
     <row r="12" ht="45" customHeight="1">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>Build CAL once, PRM once, ARCHIEVE once (Tab 03). Lanes select and configure the primitives; they do not add new runtime logic. The near-term commercial motion is in Tab 14 (non-doctrine).</t>
         </is>
@@ -2735,14 +2802,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>01 · Position</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>Where PublicLogic sits, and what it deliberately is not.</t>
         </is>
@@ -2798,7 +2865,7 @@
       </c>
     </row>
     <row r="14" ht="195" customHeight="1">
-      <c r="A14" s="11" t="inlineStr">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>"Conceptual overlap with other proof/governance efforts is evidence the design problem is real — not evidence PublicLogic has a business. Whether PublicLogic has a business is determined by customers, not by conceptual overlap."</t>
         </is>
@@ -2844,7 +2911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2854,14 +2921,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>02 · Runtime Line</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>The canonical sequence. CAL and Manifest are a gate and a precondition, not hand-off steps.</t>
         </is>
@@ -3050,17 +3117,25 @@
       </c>
     </row>
     <row r="14" ht="45" customHeight="1">
-      <c r="A14" s="11" t="inlineStr">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>Note: CAL and Manifest are a gate and a precondition, not hand-off steps. Operator phrasing — FORM opens. PRR records. CAL gates. PRM checks. VAULT governs. ARCHIEVE seals.</t>
         </is>
       </c>
     </row>
+    <row r="16" ht="60" customHeight="1">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>Bookend Rule: FORM is the Entry Surface (received → logged); PRR + VAULT + ARCHIEVE form the Repository (closed → sealed → rolled up). PJ owns those two guarantees; the middle is content-agnostic but governance-aware — every transition is wrapped by CAL.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A14:D14"/>
     <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A16:D16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3081,14 +3156,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>03 · Primitives</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>Build CAL once, PRM once, ARCHIEVE once. The OPS numbers select and configure them.</t>
         </is>
@@ -3253,7 +3328,7 @@
       </c>
     </row>
     <row r="20" ht="45" customHeight="1">
-      <c r="A20" s="11" t="inlineStr">
+      <c r="A20" s="9" t="inlineStr">
         <is>
           <t>Rule: Build CAL once, PRM once, ARCHIEVE once. The OPS numbers select and configure them.</t>
         </is>
@@ -3287,31 +3362,31 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>04 · Rulings  🔒 LOCKED</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>The four rulings are LOCKED — settled doctrine, never open questions.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>Ruling</t>
         </is>
       </c>
-      <c r="C4" s="13" t="inlineStr">
+      <c r="C4" s="14" t="inlineStr">
         <is>
           <t>Statement</t>
         </is>
@@ -3378,7 +3453,7 @@
       </c>
     </row>
     <row r="10" ht="60" customHeight="1">
-      <c r="A10" s="14" t="inlineStr">
+      <c r="A10" s="15" t="inlineStr">
         <is>
           <t>Distilled: Containers organize continuity. Leaves produce proof. Seals preserve closure. Rollups make proof visible without rewriting the parent. Module Maker authors skins, not truth.</t>
         </is>
@@ -3409,14 +3484,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>05 · CaseSpace Model</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>Type field, standing vs closing, object model, lifecycles, nesting.</t>
         </is>
@@ -3560,7 +3635,7 @@
       </c>
     </row>
     <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="11" t="inlineStr">
+      <c r="A25" s="9" t="inlineStr">
         <is>
           <t>PRM runs over Holds, never over the Subject.</t>
         </is>
@@ -3636,14 +3711,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>06 · Conflict Types</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>Conflicts never throw; they route to blocked.</t>
         </is>
@@ -3782,7 +3857,7 @@
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>Conflicts never throw; they route to blocked. Cleared only via the `resolve` transition, gated by decision_authority, itself audited.</t>
         </is>
@@ -3815,21 +3890,21 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>07 · Type Catalogue</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>The axis is proof, not cycle.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="60" customHeight="1">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>Examples and close-proof rules below are ILLUSTRATIVE — proposed, derived from the established model and from cases already named in the canon. They are not yet ratified doctrine (propose, then ratify). The type NAMES are canon; the example/proof cells are TBD until ratified.</t>
         </is>
@@ -4262,7 +4337,7 @@
       <c r="D28" s="8" t="inlineStr"/>
     </row>
     <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="11" t="inlineStr">
+      <c r="A30" s="9" t="inlineStr">
         <is>
           <t>Distinguishing rule: a leaf closes with its own proof; a container's state is the rollup of what it holds. The axis is proof, not cycle.</t>
         </is>
@@ -4296,14 +4371,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>08 · Type = Skin + Authoring Rule</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>A Type and a skin are the same artifact, two audiences.</t>
         </is>
@@ -4415,7 +4490,7 @@
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="11" t="inlineStr">
+      <c r="A15" s="9" t="inlineStr">
         <is>
           <t>Fail any of 3–6 → it is engineering, not a type; the loader rejects it.</t>
         </is>

</xml_diff>

<commit_message>
Seal Bookend doctrine with three precision corrections
Resolve three spots where the new foundational text rubbed against locked
rulings, then seal Bookend + Agnostic Middle + Runtime Contract as one
section and add PROOF.md as the spine.

- Principle #1 -> "only top-level primitive"; Owner/Subject/Resource/Window
  are parts, not peers (no longer fights the object model).
- Repository "closed -> sealed -> rollup" retyped as state -> operation ->
  view, preserving the Seals-into-parent = Rollup View ruling.
- Category -> "governed transitions between two fixed contracts: provenance
  at entry, immutability at exit" (keeps the entry/exit asymmetry).
- Add moat framing (#2 + #3 are a stance, not a feature).
- Add PROOF.md leading with the three foundational principles.
- Apply the same corrections to both workbooks (lossless xlsx edits).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VAv7tVCy2hbSMpZ9X88jpW
</commit_message>
<xml_diff>
--- a/publiclogic/docs/canon/PublicLogic-Canon.xlsx
+++ b/publiclogic/docs/canon/PublicLogic-Canon.xlsx
@@ -698,7 +698,7 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>CaseSpace is the only primitive.</t>
+          <t>CaseSpace is the only top-level primitive — the one thing that opens, moves, and seals. Owner/Subject/Resource/Window are its parts, not peers; OPS modules are presets over those parts.</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>PuddleJumper owns the two guarantees: Entry and Repository.</t>
+          <t>PuddleJumper owns the two guarantees: Entry (provenance) and Repository (immutability).</t>
         </is>
       </c>
     </row>
@@ -726,10 +726,10 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="120" customHeight="1">
+    <row r="17" ht="195" customHeight="1">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>Bookend Rule: PJ owns the Entry Surface (received → logged) and the Repository (closed → sealed → rolled up). Everything between belongs to the operator — content-agnostic, not unconstrained. Category: governed transitions between two immutable guarantees.</t>
+          <t>Bookend Rule: PJ owns the Entry Surface (received → logged) and the Repository — typed, not a state chain: PRR ends at closed (state), ARCHIEVE seals the leaf (operation), the parent renders rollup (view). The middle is content-agnostic but governance-aware. Category: governed transitions between two fixed contracts — provenance at entry, immutability at exit. The moat is principles 2 and 3 — a stance, not a feature competitors lack.</t>
         </is>
       </c>
     </row>
@@ -3123,10 +3123,10 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="60" customHeight="1">
+    <row r="16" ht="90" customHeight="1">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t>Bookend Rule: FORM is the Entry Surface (received → logged); PRR + VAULT + ARCHIEVE form the Repository (closed → sealed → rolled up). PJ owns those two guarantees; the middle is content-agnostic but governance-aware — every transition is wrapped by CAL.</t>
+          <t>Bookend Rule: FORM is the Entry Surface (received → logged, guaranteeing provenance); PRR + VAULT + ARCHIEVE form the Repository (guaranteeing immutability) — typed, not a state chain: PRR closed = state, ARCHIEVE seal = operation, parent rollup = view. PJ owns those two guarantees; the middle is content-agnostic but governance-aware — every transition is wrapped by CAL.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Pull forward old VAULT packet keepers into canon (V1.2)
Salvage the genuinely useful ideas from the original municipal-records
VAULT packet, modernized and recentered on work (records as output):
- Signal Behavior Rule (the big keeper) -> §1 doctrine + Canon Law +
  Series 1 01_Core_Doctrine: tool-agnostic intake, rule-aware behavior.
- Classification gate (four outcomes; recommend-then-ratify) -> §4.
- Record Lifecycle view (old 6-step lifecycle, kept as a view inside a
  CaseSpace, mapped to the runtime) -> §4.
- Stewardship Onboarding Track -> Appendix C (Live CaseSpace tier).
- Lineage map with refactored/retired terms (SEAL retired; CAL owns
  validation; ARCHIEVE = repository/seal) -> Appendix D + Vocabulary.
Guardrails: VAULT not reframed as records-retention; classification is
recommended, not auto-determined (counsel-ready fence intact).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VAv7tVCy2hbSMpZ9X88jpW
</commit_message>
<xml_diff>
--- a/publiclogic/docs/canon/PublicLogic-Canon.xlsx
+++ b/publiclogic/docs/canon/PublicLogic-Canon.xlsx
@@ -1012,7 +1012,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1126,6 +1126,18 @@
       <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Including about its own templates. A suggestion can never satisfy a CAL gate or drive a transition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Signal behavior</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>PJ does not care what tool produced the signal — form, email, call, upload, PMS event, calendar, invoice, photo, or spreadsheet. It cares what the signal becomes once it is a CaseSpace: a fact, a missing item, a decision, a proof event, a transitory reference, or a sealed record. Classification is recommended by rule and ratified by an authorized user — never an automated determination.</t>
         </is>
       </c>
     </row>
@@ -1728,7 +1740,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -1913,6 +1925,18 @@
         </is>
       </c>
       <c r="B22" s="18" t="inlineStr">
+        <is>
+          <t>retired — never use as a live term</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>SEAL (standalone validation tool)</t>
+        </is>
+      </c>
+      <c r="B23" s="18" t="inlineStr">
         <is>
           <t>retired — never use as a live term</t>
         </is>

</xml_diff>